<commit_message>
Add lion age, ageing reflex and lion_ages list update in Assignment_3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assignment_3/prompt_log.xlsx
+++ b/Assignment_3/prompt_log.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -590,6 +590,106 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Commit and push to GitHub</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Committed Assignment_3 (model + prompt log) as 5e9bbb4 and pushed to GitHub</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>African_Savannah_2 changes left out on purpose</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Add lion ages to the list in init; reflex removes previous and adds current age values (discussed age attribute, start age, ageing and reflex order first)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Added lion attribute int age &lt;- rnd(0, 60) and reflex grow_older (+1 per step); init loop adds all lion ages to lion_ages; global reflex update_lion_ages removes all old values and adds current ages</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Global reflex runs before lion reflexes (GAMA wiki, Runtime Concepts), so the list lags one step behind the lions' age and still contains lions that starve in that step; documented in a code comment</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Explain how the code now works</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>- (explanation only, no code change)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Explained init, step order (global reflex before lion reflexes) and the one-step lag of lion_ages with an example</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Commit and push to GitHub</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Committed Assignment_3 (model version 3.2 + prompt log) and pushed to GitHub</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Log row added before committing so the log on GitHub is complete; African_Savannah_2 changes left out</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Report lion age statistics each step in Assignment_3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assignment_3/prompt_log.xlsx
+++ b/Assignment_3/prompt_log.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -690,6 +690,56 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Each time step, report number of values in the list, their minimum, mean and maximum (console and monitors; 0 if empty; mean rounded)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>update_lion_ages now calculates count, min, mean (with_precision 1) and max of lion_ages and writes them to the console; added monitors Number of ages, Min age, Mean age, Max age</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>All values from lion_ages, so they share its one-step lag; empty list gives 0 instead of nil</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Model checked in GAMA (no warnings); commit and push to GitHub</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Committed Assignment_3 (model version 3.3 + prompt log) and pushed to GitHub</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Model compiles without warnings in GAMA 2025-06 (checked by user); African_Savannah_2 changes left out</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Colour lions by mean age and update experiment comment in Assignment_3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assignment_3/prompt_log.xlsx
+++ b/Assignment_3/prompt_log.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -740,6 +740,81 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Update the outdated comment of the experiment</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Experiment comment now also mentions the lion age monitors (number, min, mean, max)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Comment only, no change to model behaviour</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Colour lions in shades of red according to the mean age of the population (only lions, same shade for all, from the list, light red to dark red at mean age 100, replaces orange)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Added global max_mean_age_color &lt;- 100.0 and action color_lions (blends rgb(255,200,200) to rgb(120,0,0) by mean of lion_ages, asks all lions to take the shade); called in init and in update_lion_ages; lion colour starts light red instead of orange; updated aspect comment</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>All lions share one shade, so differences between lions are not visible; colour has the same one-step lag as the list; mean starts ~30, so dark red after ~70 steps</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Red shading works in GAMA; commit and push to GitHub</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Committed Assignment_3 (model version 3.4 + prompt log) and pushed to GitHub</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Lion colouring confirmed working by user; African_Savannah_2 changes left out</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Let lions die of old age after 60 years in Assignment_3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assignment_3/prompt_log.xlsx
+++ b/Assignment_3/prompt_log.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -815,6 +815,56 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Lions die if older than 60 years (1 step = 1 year; max_age in global, no slider; colour scale linked to max_age)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Added global int max_age &lt;- 60 and lion reflex die_of_old_age (when age &gt; max_age, after grow_older); max_mean_age_color now float(max_age) instead of 100; age comments changed to years; list comment now says lions that die (not only starve)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Without births all lions die within ~60 steps; lions starting at 60 die in step 1; mean age stays below 60, colour reaches dark red only if few old lions remain</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Old-age death works in GAMA; commit and push to GitHub</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Committed Assignment_3 (model version 3.5 + prompt log) and pushed to GitHub</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Model confirmed working by user; African_Savannah_2 changes left out</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add lion births on old-age death and age labels in Assignment_3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assignment_3/prompt_log.xlsx
+++ b/Assignment_3/prompt_log.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -865,6 +865,156 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Just before an old lion dies, a baby lion is born (1 per old-age death; age 0, at the old lion's place, start energy, current population shade)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>In reflex die_of_old_age: create lion number: 1 with location and color of the old lion and age 0, then do die</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Old lions are replaced 1:1, so the population only falls by starvation; babies lower the mean age and lighten the colour; babies enter lion_ages in the next step</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>What is the monitor 'Number of ages'?</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>- (explanation only, no code change)</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Monitor shows length(lion_ages) = number of values in the list; equals the number of lions at the start of the step, so it can differ from 'Number of lions' by the one-step lag</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Rename monitor 'Number of ages'</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Monitor renamed to 'Number of lions in age list'</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Label only, no change to model behaviour</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Is it possible to see the current age of each lion directly in the simulation?</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>- (question only, no code change yet)</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Options: inspect/browse agents in GAMA without code change, age as text label on each lion, or a monitor with all current ages</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Show each lion's current age on the map (option 2: text label)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Lion aspect now also draws string(age) in black bold Arial 10 next to the circle</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Shows the lion's own current age (no lag); map may look busy with many lions</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Births, monitor rename and age labels work in GAMA; commit and push to GitHub</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Committed Assignment_3 (model version 3.7 + prompt log) and pushed to GitHub</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Model confirmed working by user; African_Savannah_2 changes left out</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>